<commit_message>
feat: dialects, range-only bindings, faithful ODS dates; drop graph libraries
- Dialect (xlsx/ods, from the file extension, --dialect to force) selects
  LibreOffice vs Excel behavior for operators and coercions: 0^0, odd roots,
  booleans as numbers, direct text in SUM, number-to-text format; ods::ISNUMBER
  overrides the function. Date system 1899 (real calendar) is the ODS default.
- Inputs/outputs are lists of ranges; JSON keys are canonical range text.
- Remove petgraph and ultragraph (dev-dependencies and benchmark); the SCC
  test checks against BFS reachability.
- Depend on the sheetrs branch that numbers ODS dates from the null date and
  reads time values; ODS/XLSX parity is now exact.
- docs/FIDELITY.md lists every Excel/LibreOffice difference with its evidence;
  tests/probe.rs reproduces LibreOffice on ~120 probes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011MRBtaN4HWRL7ovwpZgUes
</commit_message>
<xml_diff>
--- a/tests/assets/semantics.xlsx
+++ b/tests/assets/semantics.xlsx
@@ -464,19 +464,19 @@
     <t xml:space="preserve">INDIRECT("Data!B"&amp;2)</t>
   </si>
   <si>
-    <t xml:space="preserve">"["&amp;TEXT(DATE(2024,1,31),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(DATE(2024,14,1),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(DATE(2024,3,0),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(DATE(1900,3,1),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(DATE(2024,2,29)+1,"0")&amp;"]"</t>
+    <t xml:space="preserve">DATE(2024,1,31)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE(2024,14,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE(2024,3,0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE(1900,3,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE(2024,2,29)+1</t>
   </si>
   <si>
     <t xml:space="preserve">YEAR(Data!C1)</t>
@@ -494,16 +494,16 @@
     <t xml:space="preserve">WEEKDAY(Data!C1,2)</t>
   </si>
   <si>
-    <t xml:space="preserve">"["&amp;TEXT(EDATE(DATE(2024,1,31),1),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(EDATE(DATE(2024,3,31),-1),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(EOMONTH(Data!C1,0),"0")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(EOMONTH(Data!C1,2),"0")&amp;"]"</t>
+    <t xml:space="preserve">EDATE(DATE(2024,1,31),1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDATE(DATE(2024,3,31),-1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOMONTH(Data!C1,0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOMONTH(Data!C1,2)</t>
   </si>
   <si>
     <t xml:space="preserve">_xlfn.DAYS(Data!C2,Data!C1)</t>
@@ -527,10 +527,10 @@
     <t xml:space="preserve">SECOND(0.7512)</t>
   </si>
   <si>
-    <t xml:space="preserve">"["&amp;TEXT(TIME(13,30,0),"0.0000")&amp;"]"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"["&amp;TEXT(DATEVALUE("2024-03-01"),"0")&amp;"]"</t>
+    <t xml:space="preserve">TIME(13,30,0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATEVALUE("2024-03-01")</t>
   </si>
   <si>
     <t xml:space="preserve">PMT(0.01,12,-1000)</t>
@@ -648,11 +648,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="0.00%"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="168" formatCode="hh:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="169" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="0.00%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -720,7 +723,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -729,11 +732,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -939,16 +958,16 @@
       <c r="B1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="0" t="n">
+      <c r="C1" s="1" t="n">
         <v>45306</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="0" t="n">
@@ -968,7 +987,7 @@
       <c r="B2" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>45338</v>
       </c>
       <c r="E2" s="0" t="n">
@@ -997,7 +1016,7 @@
       <c r="B3" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>45368</v>
       </c>
       <c r="H3" s="0" t="n">
@@ -1017,7 +1036,7 @@
       <c r="B4" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>45400</v>
       </c>
       <c r="H4" s="0" t="n">
@@ -1037,7 +1056,7 @@
       <c r="B5" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>45431</v>
       </c>
       <c r="H5" s="0" t="n">
@@ -1057,7 +1076,7 @@
       <c r="B6" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>45463</v>
       </c>
     </row>
@@ -1068,7 +1087,7 @@
       <c r="B7" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>45494</v>
       </c>
     </row>
@@ -1079,7 +1098,7 @@
       <c r="B8" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>45526</v>
       </c>
     </row>
@@ -1652,7 +1671,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="b">
+      <c r="A62" s="3" t="b">
         <f aca="false">AND(TRUE(),1,Data!A1&gt;1)</f>
         <v>1</v>
       </c>
@@ -1661,7 +1680,7 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1" t="b">
+      <c r="A63" s="3" t="b">
         <f aca="false">OR(FALSE(),0,Data!A1&lt;1)</f>
         <v>0</v>
       </c>
@@ -1670,7 +1689,7 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1" t="b">
+      <c r="A64" s="3" t="b">
         <f aca="false">NOT(Data!A1&gt;1)</f>
         <v>0</v>
       </c>
@@ -1679,7 +1698,7 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1" t="b">
+      <c r="A65" s="3" t="b">
         <f aca="false">_xlfn.XOR(TRUE(),TRUE())</f>
         <v>0</v>
       </c>
@@ -1715,7 +1734,7 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="1" t="b">
+      <c r="A69" s="3" t="b">
         <f aca="false">ISNUMBER(Data!A1)</f>
         <v>1</v>
       </c>
@@ -1724,7 +1743,7 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="1" t="b">
+      <c r="A70" s="3" t="b">
         <f aca="false">ISTEXT(Data!B1)</f>
         <v>1</v>
       </c>
@@ -1733,7 +1752,7 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="1" t="b">
+      <c r="A71" s="3" t="b">
         <f aca="false">ISBLANK(Data!B9)</f>
         <v>1</v>
       </c>
@@ -1742,7 +1761,7 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="1" t="b">
+      <c r="A72" s="3" t="b">
         <f aca="false">ISERROR(1/0)</f>
         <v>1</v>
       </c>
@@ -1751,7 +1770,7 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="b">
+      <c r="A73" s="3" t="b">
         <f aca="false">ISNA(NA())</f>
         <v>1</v>
       </c>
@@ -1760,7 +1779,7 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="1" t="b">
+      <c r="A74" s="3" t="b">
         <f aca="false">ISEVEN(4)</f>
         <v>1</v>
       </c>
@@ -1769,7 +1788,7 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="1" t="b">
+      <c r="A75" s="3" t="b">
         <f aca="false">ISODD(4)</f>
         <v>0</v>
       </c>
@@ -1778,7 +1797,7 @@
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="1" t="b">
+      <c r="A76" s="3" t="b">
         <f aca="false">ISLOGICAL(TRUE())</f>
         <v>1</v>
       </c>
@@ -1931,7 +1950,7 @@
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="1" t="b">
+      <c r="A93" s="3" t="b">
         <f aca="false">EXACT("a","A")</f>
         <v>0</v>
       </c>
@@ -2228,7 +2247,7 @@
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="0" t="n">
+      <c r="A126" s="1" t="n">
         <f aca="false">SUM(INDEX(Data!A1:C8,2,0))</f>
         <v>45341</v>
       </c>
@@ -2354,45 +2373,45 @@
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(DATE(2024,1,31),"0")&amp;"]"</f>
-        <v>[45322]</v>
+      <c r="A140" s="4" t="n">
+        <f aca="false">DATE(2024,1,31)</f>
+        <v>45322</v>
       </c>
       <c r="B140" s="0" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(DATE(2024,14,1),"0")&amp;"]"</f>
-        <v>[45689]</v>
+      <c r="A141" s="4" t="n">
+        <f aca="false">DATE(2024,14,1)</f>
+        <v>45689</v>
       </c>
       <c r="B141" s="0" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(DATE(2024,3,0),"0")&amp;"]"</f>
-        <v>[45351]</v>
+      <c r="A142" s="4" t="n">
+        <f aca="false">DATE(2024,3,0)</f>
+        <v>45351</v>
       </c>
       <c r="B142" s="0" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(DATE(1900,3,1),"0")&amp;"]"</f>
-        <v>[61]</v>
+      <c r="A143" s="4" t="n">
+        <f aca="false">DATE(1900,3,1)</f>
+        <v>61</v>
       </c>
       <c r="B143" s="0" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(DATE(2024,2,29)+1,"0")&amp;"]"</f>
-        <v>[45352]</v>
+      <c r="A144" s="4" t="n">
+        <f aca="false">DATE(2024,2,29)+1</f>
+        <v>45352</v>
       </c>
       <c r="B144" s="0" t="s">
         <v>151</v>
@@ -2444,36 +2463,36 @@
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(EDATE(DATE(2024,1,31),1),"0")&amp;"]"</f>
-        <v>[45351]</v>
+      <c r="A150" s="0" t="n">
+        <f aca="false">EDATE(DATE(2024,1,31),1)</f>
+        <v>45351</v>
       </c>
       <c r="B150" s="0" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(EDATE(DATE(2024,3,31),-1),"0")&amp;"]"</f>
-        <v>[45351]</v>
+      <c r="A151" s="0" t="n">
+        <f aca="false">EDATE(DATE(2024,3,31),-1)</f>
+        <v>45351</v>
       </c>
       <c r="B151" s="0" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(EOMONTH(Data!C1,0),"0")&amp;"]"</f>
-        <v>[45322]</v>
+      <c r="A152" s="0" t="n">
+        <f aca="false">EOMONTH(Data!C1,0)</f>
+        <v>45322</v>
       </c>
       <c r="B152" s="0" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(EOMONTH(Data!C1,2),"0")&amp;"]"</f>
-        <v>[45382]</v>
+      <c r="A153" s="0" t="n">
+        <f aca="false">EOMONTH(Data!C1,2)</f>
+        <v>45382</v>
       </c>
       <c r="B153" s="0" t="s">
         <v>160</v>
@@ -2543,25 +2562,25 @@
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(TIME(13,30,0),"0.0000")&amp;"]"</f>
-        <v>[0.5625]</v>
+      <c r="A161" s="5" t="n">
+        <f aca="false">TIME(13,30,0)</f>
+        <v>0.5625</v>
       </c>
       <c r="B161" s="0" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="0" t="str">
-        <f aca="false">"["&amp;TEXT(DATEVALUE("2024-03-01"),"0")&amp;"]"</f>
-        <v>[45352]</v>
+      <c r="A162" s="0" t="n">
+        <f aca="false">DATEVALUE("2024-03-01")</f>
+        <v>45352</v>
       </c>
       <c r="B162" s="0" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="6" t="n">
         <f aca="false">PMT(0.01,12,-1000)</f>
         <v>88.8487886783417</v>
       </c>
@@ -2570,7 +2589,7 @@
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="6" t="n">
         <f aca="false">PMT(0.05/12,360,200000)</f>
         <v>-1073.64324602428</v>
       </c>
@@ -2579,7 +2598,7 @@
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="6" t="n">
         <f aca="false">FV(0.05,10,-100)</f>
         <v>1257.78925355488</v>
       </c>
@@ -2588,7 +2607,7 @@
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="6" t="n">
         <f aca="false">PV(0.05,10,-100)</f>
         <v>772.173492918482</v>
       </c>
@@ -2597,7 +2616,7 @@
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="6" t="n">
         <f aca="false">NPV(0.1,100,200,300)</f>
         <v>481.592787377911</v>
       </c>
@@ -2606,7 +2625,7 @@
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="3" t="n">
+      <c r="A168" s="7" t="n">
         <f aca="false">IRR(Data!J1:J5)</f>
         <v>0.248883356624071</v>
       </c>
@@ -2678,7 +2697,7 @@
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="1" t="b">
+      <c r="A176" s="3" t="b">
         <f aca="false">1="1"</f>
         <v>0</v>
       </c>
@@ -2687,7 +2706,7 @@
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="1" t="b">
+      <c r="A177" s="3" t="b">
         <f aca="false">"a"&lt;"B"</f>
         <v>1</v>
       </c>
@@ -2696,7 +2715,7 @@
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="1" t="b">
+      <c r="A178" s="3" t="b">
         <f aca="false">"abc"="ABC"</f>
         <v>1</v>
       </c>
@@ -2705,7 +2724,7 @@
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="1" t="b">
+      <c r="A179" s="3" t="b">
         <f aca="false">1&lt;"a"</f>
         <v>1</v>
       </c>
@@ -2885,7 +2904,7 @@
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A199" s="1" t="b">
+      <c r="A199" s="3" t="b">
         <f aca="false">ISERROR(Data!A1/0)</f>
         <v>1</v>
       </c>

</xml_diff>